<commit_message>
docs(balance): record founder monetization decision — boosters IAP + rewarded ads
Founder selection 2026-07-18: consumable boosters (IAP) and rewarded-ads
hybrid, combined. Recorded in game-concept.md §Monetization and the
workbook tab (renamed 'Monetization DIRECTION', selected rows marked).

Binding follow-ups captured in both places:
- Phase 2: monetization GDD co-designed with booster-brewing.md as ONE
  task — earned brewing loop stays primary, paid boosters must never
  obsolete brewed ones
- Rewarded-ad placements require ux-review sign-off
- Ad-mediation SDK selection = future ADR
- Anti-pillars unchanged: no guaranteed-completion sales, no pay-to-win

Design doc: design/gdd/game-concept.md

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EzxVYzM8MpTaRR6pfEZowd
</commit_message>
<xml_diff>
--- a/design/balance/sweet-cascade-economy-v1.xlsx
+++ b/design/balance/sweet-cascade-economy-v1.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Level Balance" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Star Economy" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Brewing P2 DRAFT" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Monetization NOT DESIGNED" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Monetization DIRECTION" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47,7 +47,7 @@
       <color rgb="000000FF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -62,6 +62,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -91,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -111,6 +117,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2073,7 +2080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2084,9 +2091,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Monetization — NOT DESIGNED (deliberate). Frames the future decision; contains no design.</t>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Monetization — DIRECTION CHOSEN (founder, 2026-07-18): consumable boosters (IAP) + rewarded-ads hybrid, COMBINED. Detailed design remains Phase 2, gated on co-design with booster-brewing.md (earned loop stays primary).</t>
         </is>
       </c>
     </row>
@@ -2123,6 +2130,11 @@
           <t>Genre precedent</t>
         </is>
       </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Founder decision (2026-07-18)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
@@ -2150,6 +2162,11 @@
           <t>Rare in match-3; common elsewhere</t>
         </is>
       </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>NOT selected (may return later as add-on)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
@@ -2177,6 +2194,11 @@
           <t>Candy Crush / Royal Match core model</t>
         </is>
       </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>SELECTED — Phase 2 design, must reconcile with earned brewing loop</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="40" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
@@ -2204,6 +2226,11 @@
           <t>Royal Match, most modern match-3</t>
         </is>
       </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>NOT selected (needs events engine, Phase 3 — revisit then)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
@@ -2229,6 +2256,18 @@
       <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Common in casual</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>SELECTED — Phase 2 design, placement UX + mediation SDK (future ADR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Binding follow-ups: (1) booster-brewing.md (Phase 2) and the monetization GDD are ONE design task — paid boosters must never obsolete brewed ones; (2) rewarded-ad placements need UX-review sign-off (session-flow guardrail); (3) ad-mediation SDK choice = future ADR; (4) anti-pillars unchanged: no guaranteed-completion sales, no pay-to-win stars.</t>
         </is>
       </c>
     </row>

</xml_diff>